<commit_message>
Finalize Level 2 lessons 2.1-2.6 (reviewed and verified)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GVxwagJ2ocBAdfHuqZnXCC
</commit_message>
<xml_diff>
--- a/02-formulas-functions/04-math-statistical-functions/2.4-math-statistical-functions.xlsx
+++ b/02-formulas-functions/04-math-statistical-functions/2.4-math-statistical-functions.xlsx
@@ -1084,10 +1084,10 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="49" customHeight="1">
+    <row r="2" ht="64" customHeight="1">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>Tasks use three data sheets. Stays holds 573 inpatient stays (rows 2–574), ED holds 785 visits (rows 2–786), and Meds holds 388 medication orders (rows 2–389). Reference a column's data rows, like Stays!J2:J574, rather than a whole column like J:J, because the header text in row 1 breaks the row-by-row math in SUMPRODUCT. When a task asks you to round, round with a function so the stored value matches, not just the display.</t>
+          <t>Tasks use three data sheets. Stays holds 573 inpatient stays (rows 2–574), ED holds 785 visits (rows 2–786), and Meds holds 388 medication orders (rows 2–389). Reference a column's data rows, like Stays!J2:J574, rather than a whole column like J:J, because the header text in row 1 breaks the row-by-row math in SUMPRODUCT. Structured references such as tblStays[TotalCharges] work too. When a task asks you to round, round with a function so the stored value matches, not just the display.</t>
         </is>
       </c>
     </row>
@@ -1197,7 +1197,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" ht="66" customHeight="1">
+    <row r="9" ht="81" customHeight="1">
       <c r="A9" s="18" t="inlineStr">
         <is>
           <t>4</t>
@@ -1205,12 +1205,12 @@
       </c>
       <c r="B9" s="19" t="inlineStr">
         <is>
-          <t>ED leaders review the three longest ED stays each period for boarding delays. They report each stay in whole hours and count any started hour as a full hour. Find the 3rd-longest EDLOSMin on the ED sheet, convert it to hours, and round it up to a whole number of hours with ROUNDUP.</t>
+          <t>ED leaders review the three longest ED visits for boarding delays, where an admitted patient waits in the ED for an inpatient bed. They report each visit's length of stay in whole hours and count any started hour as a full hour. Find the 3rd-longest EDLOSMin on the ED sheet, convert it to hours, and round it up to a whole number of hours with ROUNDUP.</t>
         </is>
       </c>
       <c r="C9" s="20" t="inlineStr">
         <is>
-          <t>LARGE(array, k) finds the stay. Divide by 60, then ROUNDUP(…, 0)</t>
+          <t>LARGE(array, k) finds the visit. Divide by 60, then ROUNDUP(…, 0)</t>
         </is>
       </c>
       <c r="D9" s="21" t="n"/>
@@ -1329,7 +1329,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" ht="51" customHeight="1">
+    <row r="15" ht="81" customHeight="1">
       <c r="A15" s="18" t="inlineStr">
         <is>
           <t>10</t>
@@ -1337,7 +1337,7 @@
       </c>
       <c r="B15" s="19" t="inlineStr">
         <is>
-          <t>Fill the yellow AgeBand column on the Stays sheet with each stay's 10-year age band using FLOOR.MATH, so age 78 becomes 70 and age 80 becomes 80. Start in K2. The gray cell counts the stays in the 80–89 band.</t>
+          <t>Fill the yellow AgeBand column on the Stays sheet with each stay's 10-year age band using FLOOR.MATH, so age 78 becomes 70 and age 80 becomes 80. Type the formula in K2. Stays is an Excel Table, so Excel fills the formula down the whole column for you. If it doesn't, double-click the fill handle. The gray cell counts the stays in the 80–89 band.</t>
         </is>
       </c>
       <c r="C15" s="20" t="inlineStr">
@@ -1362,17 +1362,17 @@
       </c>
       <c r="B16" s="19" t="inlineStr">
         <is>
-          <t>The ED status board rounds each visit's length of stay to the nearest 15 minutes and shows it as hours and minutes, like "6 h 45 min". What does it show for visit ED211176 (ED row 2, EDLOSMin = 624)? Build the text with one formula that refers to the EDLOSMin cell.</t>
+          <t>Order RX824601 (Meds row 255) is vancomycin 1,250 mg every 12 hours, with 24 doses dispensed. Assume the IV room mixes every dose from 500 mg single-dose vials and throws away whatever is left in an opened vial. How many vials did this order use?</t>
         </is>
       </c>
       <c r="C16" s="20" t="inlineStr">
         <is>
-          <t>MROUND to 15 first. Then INT(minutes/60) gives hours and MOD(minutes,60) gives the minutes left over. Join with &amp;</t>
-        </is>
-      </c>
-      <c r="D16" s="26" t="n"/>
+          <t>Work out vials per dose first: round 1,250 mg UP to a whole number of 500 mg vials with CEILING.MATH (or ROUNDUP)</t>
+        </is>
+      </c>
+      <c r="D16" s="21" t="n"/>
       <c r="E16" s="22">
-        <f>IF(IFERROR(D16="",FALSE),"",IF(IFERROR(OR(LOWER(TRIM(D16&amp;""))=LOWER(TRIM('Answer Key'!$C$15&amp;"")),LOWER(TRIM(D16&amp;""))="10h 30min",LOWER(TRIM(D16&amp;""))="10h30min",LOWER(TRIM(D16&amp;""))="10 h 30 m",LOWER(TRIM(D16&amp;""))="10h 30m",LOWER(TRIM(D16&amp;""))="10h30m",LOWER(TRIM(D16&amp;""))="10 hr 30 min",LOWER(TRIM(D16&amp;""))="10 h 30 mins",LOWER(TRIM(D16&amp;""))="10 hrs 30 min"),FALSE),"✔ Correct","✘ Not yet"))</f>
+        <f>IF(IFERROR(D16="",FALSE),"",IF(IFERROR(AND(ISNUMBER(D16),OR(ABS(D16-'Answer Key'!$C$15)&lt;=0.0001)),FALSE),"✔ Correct","✘ Not yet"))</f>
         <v/>
       </c>
     </row>
@@ -1406,17 +1406,17 @@
       </c>
       <c r="B18" s="19" t="inlineStr">
         <is>
-          <t>Order RX824601 (Meds row 255) is vancomycin 1,250 mg every 12 hours, with 24 doses dispensed. Assume the IV room mixes every dose from 500 mg single-dose vials and throws away whatever is left in an opened vial. How many vials did this order use?</t>
+          <t>The ED status board rounds each visit's length of stay to the nearest 15 minutes and shows it as hours and minutes, like "6 h 45 min". What does it show for visit ED211176 (ED row 2, EDLOSMin = 624)? Build the text with one formula that refers to the EDLOSMin cell.</t>
         </is>
       </c>
       <c r="C18" s="20" t="inlineStr">
         <is>
-          <t>Work out vials per dose first: round 1,250 mg UP to a whole number of 500 mg vials with CEILING.MATH (or ROUNDUP)</t>
-        </is>
-      </c>
-      <c r="D18" s="21" t="n"/>
+          <t>MROUND to 15 first. Then INT(minutes/60) gives hours and MOD(minutes,60) gives the minutes left over. Join with &amp;</t>
+        </is>
+      </c>
+      <c r="D18" s="26" t="n"/>
       <c r="E18" s="22">
-        <f>IF(IFERROR(D18="",FALSE),"",IF(IFERROR(AND(ISNUMBER(D18),OR(ABS(D18-'Answer Key'!$C$17)&lt;=0.0001)),FALSE),"✔ Correct","✘ Not yet"))</f>
+        <f>IF(IFERROR(D18="",FALSE),"",IF(IFERROR(OR(LOWER(TRIM(D18&amp;""))=LOWER(TRIM('Answer Key'!$C$17&amp;"")),LOWER(TRIM(D18&amp;""))="10h 30min",LOWER(TRIM(D18&amp;""))="10h30min",LOWER(TRIM(D18&amp;""))="10 h 30 m",LOWER(TRIM(D18&amp;""))="10h 30m",LOWER(TRIM(D18&amp;""))="10h30m",LOWER(TRIM(D18&amp;""))="10 hr 30 min",LOWER(TRIM(D18&amp;""))="10 h 30 mins",LOWER(TRIM(D18&amp;""))="10 hrs 30 min"),FALSE),"✔ Correct","✘ Not yet"))</f>
         <v/>
       </c>
     </row>
@@ -68072,7 +68072,7 @@
       </c>
       <c r="B8" s="19" t="inlineStr">
         <is>
-          <t>ED leaders review the three longest ED stays each period for boarding delays. They report each stay in whole hours and count any started hour as a full hour. Find the 3rd-longest EDLOSMin on the ED sheet, convert it to hours, and round it up to a whole number of hours with ROUNDUP.</t>
+          <t>ED leaders review the three longest ED visits for boarding delays, where an admitted patient waits in the ED for an inpatient bed. They report each visit's length of stay in whole hours and count any started hour as a full hour. Find the 3rd-longest EDLOSMin on the ED sheet, convert it to hours, and round it up to a whole number of hours with ROUNDUP.</t>
         </is>
       </c>
       <c r="C8" s="38" t="n">
@@ -68089,7 +68089,7 @@
       </c>
       <c r="F8" s="19" t="inlineStr">
         <is>
-          <t>LARGE returns the k-th largest value, so LARGE(range,1) is the same as MAX. The three longest stays were 1,304, 1,281, and 1,169 minutes. The 3rd is 1,169 ÷ 60 = 19.48 hours, and ROUNDUP turns the started hour into a full one, giving 20. ROUND and ROUNDDOWN both give 19 here, which would under-report the stay because the rule counts every started hour. =CEILING.MATH(LARGE(…,3)/60) gives the same 20. Change k to 2 or 1 to list the other two stays.</t>
+          <t>LARGE returns the k-th largest value, so LARGE(range,1) is the same as MAX. The three longest visits lasted 1,304, 1,281, and 1,169 minutes. The 3rd is 1,169 ÷ 60 = 19.48 hours, and ROUNDUP turns the started hour into a full one, giving 20. ROUND and ROUNDDOWN both give 19 here, which would under-report the visit because the rule counts every started hour. =CEILING.MATH(LARGE(…,3)/60) gives the same 20. Change k to 2 or 1 to see the other two visits.</t>
         </is>
       </c>
     </row>
@@ -68238,7 +68238,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="96" customHeight="1">
+    <row r="14" ht="111" customHeight="1">
       <c r="A14" s="18" t="inlineStr">
         <is>
           <t>10</t>
@@ -68246,7 +68246,7 @@
       </c>
       <c r="B14" s="19" t="inlineStr">
         <is>
-          <t>Fill the yellow AgeBand column on the Stays sheet with each stay's 10-year age band using FLOOR.MATH, so age 78 becomes 70 and age 80 becomes 80. Start in K2. The gray cell counts the stays in the 80–89 band.</t>
+          <t>Fill the yellow AgeBand column on the Stays sheet with each stay's 10-year age band using FLOOR.MATH, so age 78 becomes 70 and age 80 becomes 80. Type the formula in K2. Stays is an Excel Table, so Excel fills the formula down the whole column for you. If it doesn't, double-click the fill handle. The gray cell counts the stays in the 80–89 band.</t>
         </is>
       </c>
       <c r="C14" s="38" t="n">
@@ -68267,7 +68267,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="96" customHeight="1">
+    <row r="15" ht="126" customHeight="1">
       <c r="A15" s="18" t="inlineStr">
         <is>
           <t>11</t>
@@ -68275,26 +68275,24 @@
       </c>
       <c r="B15" s="19" t="inlineStr">
         <is>
-          <t>The ED status board rounds each visit's length of stay to the nearest 15 minutes and shows it as hours and minutes, like "6 h 45 min". What does it show for visit ED211176 (ED row 2, EDLOSMin = 624)? Build the text with one formula that refers to the EDLOSMin cell.</t>
-        </is>
-      </c>
-      <c r="C15" s="38" t="inlineStr">
-        <is>
-          <t>10 h 30 min</t>
-        </is>
+          <t>Order RX824601 (Meds row 255) is vancomycin 1,250 mg every 12 hours, with 24 doses dispensed. Assume the IV room mixes every dose from 500 mg single-dose vials and throws away whatever is left in an opened vial. How many vials did this order use?</t>
+        </is>
+      </c>
+      <c r="C15" s="38" t="n">
+        <v>72</v>
       </c>
       <c r="D15" s="39" t="inlineStr">
         <is>
-          <t>=INT(MROUND(ED!H2,15)/60)&amp;" h "&amp;MOD(MROUND(ED!H2,15),60)&amp;" min"</t>
+          <t>=CEILING.MATH(1250,500)/500*Meds!H255</t>
         </is>
       </c>
       <c r="E15" cm="1" s="40">
-        <f t="array" ref="E15">INT(MROUND(ED!H2,15)/60)&amp;" h "&amp;MOD(MROUND(ED!H2,15),60)&amp;" min"</f>
+        <f t="array" ref="E15">_xlfn.CEILING.MATH(1250,500)/500*Meds!H255</f>
         <v/>
       </c>
       <c r="F15" s="19" t="inlineStr">
         <is>
-          <t>MROUND(624,15) returns 630, because 624 is closer to 630 than to 615. Then INT(630/60) is 10 whole hours and MOD(630,60) is the 30 minutes left over. The &amp; operator joins the pieces into "10 h 30 min". Without the rounding the board would show "10 h 24 min". TRUNC or ROUNDDOWN(…,0) can replace INT here because the minutes are positive.</t>
+          <t>CEILING.MATH(1250,500) rounds up to 1,500 mg, which is 3 vials per dose. Two vials would hold only 1,000 mg, so ROUNDDOWN would under-dose. 3 vials × 24 doses = 72 vials. Rounding the order's total instead (CEILING.MATH(1250*24,500)/500 = 60) assumes leftover drug carries over to the next dose, which a single-dose vial doesn't allow. =ROUNDUP(1250/500,0)*Meds!H255 also works. The order wasted 6,000 mg in partly used vials.</t>
         </is>
       </c>
     </row>
@@ -68323,11 +68321,11 @@
       </c>
       <c r="F16" s="19" t="inlineStr">
         <is>
-          <t>Subtracting the two columns gives each stay's variance, which is negative when the stay was shorter than expected. ABS turns every variance into a distance, the comparison turns each distance into TRUE or FALSE, -- turns those into 1s and 0s, and SUMPRODUCT adds them. Without ABS, every stay that ended early would count as on target, and you'd get 348. A helper column of =ABS(I2-H2) counted with COUNTIF(range,"&lt;=1") gives the same 264.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="126" customHeight="1">
+          <t>Subtracting the two columns gives each stay's difference from expected, which is negative when the stay was shorter than expected. ABS turns every difference into a distance, the comparison turns each distance into TRUE or FALSE, -- turns those into 1s and 0s, and SUMPRODUCT adds them. Without ABS, every stay that ended early would count as on target, and you'd get 348. A helper column of =ABS(I2-H2) counted with COUNTIF(range,"&lt;=1") gives the same 264.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="96" customHeight="1">
       <c r="A17" s="18" t="inlineStr">
         <is>
           <t>13</t>
@@ -68335,24 +68333,26 @@
       </c>
       <c r="B17" s="19" t="inlineStr">
         <is>
-          <t>Order RX824601 (Meds row 255) is vancomycin 1,250 mg every 12 hours, with 24 doses dispensed. Assume the IV room mixes every dose from 500 mg single-dose vials and throws away whatever is left in an opened vial. How many vials did this order use?</t>
-        </is>
-      </c>
-      <c r="C17" s="38" t="n">
-        <v>72</v>
+          <t>The ED status board rounds each visit's length of stay to the nearest 15 minutes and shows it as hours and minutes, like "6 h 45 min". What does it show for visit ED211176 (ED row 2, EDLOSMin = 624)? Build the text with one formula that refers to the EDLOSMin cell.</t>
+        </is>
+      </c>
+      <c r="C17" s="38" t="inlineStr">
+        <is>
+          <t>10 h 30 min</t>
+        </is>
       </c>
       <c r="D17" s="39" t="inlineStr">
         <is>
-          <t>=CEILING.MATH(1250,500)/500*Meds!H255</t>
+          <t>=INT(MROUND(ED!H2,15)/60)&amp;" h "&amp;MOD(MROUND(ED!H2,15),60)&amp;" min"</t>
         </is>
       </c>
       <c r="E17" cm="1" s="40">
-        <f t="array" ref="E17">_xlfn.CEILING.MATH(1250,500)/500*Meds!H255</f>
+        <f t="array" ref="E17">INT(MROUND(ED!H2,15)/60)&amp;" h "&amp;MOD(MROUND(ED!H2,15),60)&amp;" min"</f>
         <v/>
       </c>
       <c r="F17" s="19" t="inlineStr">
         <is>
-          <t>CEILING.MATH(1250,500) rounds up to 1,500 mg, which is 3 vials per dose. Two vials would hold only 1,000 mg, so ROUNDDOWN would under-dose. 3 vials × 24 doses = 72 vials. Rounding the order's total instead (CEILING.MATH(1250*24,500)/500 = 60) assumes leftover drug carries over to the next dose, which a single-dose vial doesn't allow. =ROUNDUP(1250/500,0)*Meds!H255 also works. The order wasted 6,000 mg in partly used vials.</t>
+          <t>MROUND(624,15) returns 630, because 624 is closer to 630 than to 615. Then INT(630/60) is 10 whole hours and MOD(630,60) is the 30 minutes left over. The &amp; operator joins the pieces into "10 h 30 min". Without the rounding the board would show "10 h 24 min". TRUNC or ROUNDDOWN(…,0) can replace INT here because the minutes are positive.</t>
         </is>
       </c>
     </row>

</xml_diff>